<commit_message>
sysid_gimbal.xlsx: regenerado con la derivada CAUSAL en 'datos_prbs_rate'
El export venia fallando con PermissionError (el .xlsx estaba abierto en Excel) y el
fallo quedo oculto tras un /dev/null, asi que la hoja seguia con la derivada central.
Con Excel cerrado, regenerado y VERIFICADO: la salida arranca en 0.0 (causal) y el
modelo del usuario vuelve a ajustar mejor con u[k-1], que es el retardo real medido.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/neo_control/sysid_gimbal.xlsx
+++ b/tools/neo_control/sysid_gimbal.xlsx
@@ -33830,7 +33830,7 @@
         <v>15.65</v>
       </c>
       <c r="C2" t="n">
-        <v>5.6814</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -33841,7 +33841,7 @@
         <v>15.65</v>
       </c>
       <c r="C3" t="n">
-        <v>8.0381</v>
+        <v>5.6814</v>
       </c>
     </row>
     <row r="4">
@@ -33852,7 +33852,7 @@
         <v>15.65</v>
       </c>
       <c r="C4" t="n">
-        <v>11.9343</v>
+        <v>10.3948</v>
       </c>
     </row>
     <row r="5">
@@ -33863,7 +33863,7 @@
         <v>15.65</v>
       </c>
       <c r="C5" t="n">
-        <v>14.7817</v>
+        <v>13.4738</v>
       </c>
     </row>
     <row r="6">
@@ -33874,7 +33874,7 @@
         <v>15.65</v>
       </c>
       <c r="C6" t="n">
-        <v>15.4046</v>
+        <v>16.0896</v>
       </c>
     </row>
     <row r="7">
@@ -33885,7 +33885,7 @@
         <v>15.65</v>
       </c>
       <c r="C7" t="n">
-        <v>15.1646</v>
+        <v>14.7196</v>
       </c>
     </row>
     <row r="8">
@@ -33896,7 +33896,7 @@
         <v>15.65</v>
       </c>
       <c r="C8" t="n">
-        <v>15.1175</v>
+        <v>15.6096</v>
       </c>
     </row>
     <row r="9">
@@ -33907,7 +33907,7 @@
         <v>15.65</v>
       </c>
       <c r="C9" t="n">
-        <v>15.8747</v>
+        <v>14.6253</v>
       </c>
     </row>
     <row r="10">
@@ -33918,7 +33918,7 @@
         <v>15.65</v>
       </c>
       <c r="C10" t="n">
-        <v>15.9055</v>
+        <v>17.1241</v>
       </c>
     </row>
     <row r="11">
@@ -33929,7 +33929,7 @@
         <v>15.65</v>
       </c>
       <c r="C11" t="n">
-        <v>15.1488</v>
+        <v>14.6869</v>
       </c>
     </row>
     <row r="12">
@@ -33940,7 +33940,7 @@
         <v>15.65</v>
       </c>
       <c r="C12" t="n">
-        <v>15.5834</v>
+        <v>15.6106</v>
       </c>
     </row>
     <row r="13">
@@ -33951,7 +33951,7 @@
         <v>15.65</v>
       </c>
       <c r="C13" t="n">
-        <v>15.3801</v>
+        <v>15.5561</v>
       </c>
     </row>
     <row r="14">
@@ -33962,7 +33962,7 @@
         <v>15.65</v>
       </c>
       <c r="C14" t="n">
-        <v>15.433</v>
+        <v>15.2041</v>
       </c>
     </row>
     <row r="15">
@@ -33973,7 +33973,7 @@
         <v>15.65</v>
       </c>
       <c r="C15" t="n">
-        <v>15.6517</v>
+        <v>15.6619</v>
       </c>
     </row>
     <row r="16">
@@ -33984,7 +33984,7 @@
         <v>15.65</v>
       </c>
       <c r="C16" t="n">
-        <v>15.2026</v>
+        <v>15.6415</v>
       </c>
     </row>
     <row r="17">
@@ -33995,7 +33995,7 @@
         <v>15.65</v>
       </c>
       <c r="C17" t="n">
-        <v>15.1919</v>
+        <v>14.7638</v>
       </c>
     </row>
     <row r="18">
@@ -34006,7 +34006,7 @@
         <v>15.65</v>
       </c>
       <c r="C18" t="n">
-        <v>16.2378</v>
+        <v>15.62</v>
       </c>
     </row>
     <row r="19">
@@ -34017,7 +34017,7 @@
         <v>15.65</v>
       </c>
       <c r="C19" t="n">
-        <v>15.992</v>
+        <v>16.8555</v>
       </c>
     </row>
     <row r="20">
@@ -34028,7 +34028,7 @@
         <v>15.65</v>
       </c>
       <c r="C20" t="n">
-        <v>15.3946</v>
+        <v>15.1286</v>
       </c>
     </row>
     <row r="21">
@@ -34039,7 +34039,7 @@
         <v>15.65</v>
       </c>
       <c r="C21" t="n">
-        <v>15.1722</v>
+        <v>15.6606</v>
       </c>
     </row>
     <row r="22">
@@ -34050,7 +34050,7 @@
         <v>15.65</v>
       </c>
       <c r="C22" t="n">
-        <v>13.3313</v>
+        <v>14.6839</v>
       </c>
     </row>
     <row r="23">
@@ -34061,7 +34061,7 @@
         <v>-15.65</v>
       </c>
       <c r="C23" t="n">
-        <v>6.6287</v>
+        <v>11.9787</v>
       </c>
     </row>
     <row r="24">
@@ -34072,7 +34072,7 @@
         <v>-15.65</v>
       </c>
       <c r="C24" t="n">
-        <v>-4.6045</v>
+        <v>1.2786</v>
       </c>
     </row>
     <row r="25">
@@ -34083,7 +34083,7 @@
         <v>-15.65</v>
       </c>
       <c r="C25" t="n">
-        <v>-10.6385</v>
+        <v>-10.4875</v>
       </c>
     </row>
     <row r="26">
@@ -34094,7 +34094,7 @@
         <v>-15.65</v>
       </c>
       <c r="C26" t="n">
-        <v>-12.1592</v>
+        <v>-10.7896</v>
       </c>
     </row>
     <row r="27">
@@ -34105,7 +34105,7 @@
         <v>-15.65</v>
       </c>
       <c r="C27" t="n">
-        <v>-14.0681</v>
+        <v>-13.5288</v>
       </c>
     </row>
     <row r="28">
@@ -34116,7 +34116,7 @@
         <v>-15.65</v>
       </c>
       <c r="C28" t="n">
-        <v>-15.82</v>
+        <v>-14.6074</v>
       </c>
     </row>
     <row r="29">
@@ -34127,7 +34127,7 @@
         <v>-15.65</v>
       </c>
       <c r="C29" t="n">
-        <v>-15.925</v>
+        <v>-17.0326</v>
       </c>
     </row>
     <row r="30">
@@ -34138,7 +34138,7 @@
         <v>-15.65</v>
       </c>
       <c r="C30" t="n">
-        <v>-15.2353</v>
+        <v>-14.8174</v>
       </c>
     </row>
     <row r="31">
@@ -34149,7 +34149,7 @@
         <v>-15.65</v>
       </c>
       <c r="C31" t="n">
-        <v>-15.6703</v>
+        <v>-15.6533</v>
       </c>
     </row>
     <row r="32">
@@ -34160,7 +34160,7 @@
         <v>-15.65</v>
       </c>
       <c r="C32" t="n">
-        <v>-15.7979</v>
+        <v>-15.6873</v>
       </c>
     </row>
     <row r="33">
@@ -34171,7 +34171,7 @@
         <v>-15.65</v>
       </c>
       <c r="C33" t="n">
-        <v>-15.9193</v>
+        <v>-15.9084</v>
       </c>
     </row>
     <row r="34">
@@ -34182,7 +34182,7 @@
         <v>-15.65</v>
       </c>
       <c r="C34" t="n">
-        <v>-15.3464</v>
+        <v>-15.9301</v>
       </c>
     </row>
     <row r="35">
@@ -34193,7 +34193,7 @@
         <v>-15.65</v>
       </c>
       <c r="C35" t="n">
-        <v>-14.7415</v>
+        <v>-14.7627</v>
       </c>
     </row>
     <row r="36">
@@ -34204,7 +34204,7 @@
         <v>-15.65</v>
       </c>
       <c r="C36" t="n">
-        <v>-15.5428</v>
+        <v>-14.7203</v>
       </c>
     </row>
     <row r="37">
@@ -34215,7 +34215,7 @@
         <v>-15.65</v>
       </c>
       <c r="C37" t="n">
-        <v>-16.4301</v>
+        <v>-16.3653</v>
       </c>
     </row>
     <row r="38">
@@ -34226,7 +34226,7 @@
         <v>-15.65</v>
       </c>
       <c r="C38" t="n">
-        <v>-15.5485</v>
+        <v>-16.4948</v>
       </c>
     </row>
     <row r="39">
@@ -34237,7 +34237,7 @@
         <v>-15.65</v>
       </c>
       <c r="C39" t="n">
-        <v>-15.1505</v>
+        <v>-14.6022</v>
       </c>
     </row>
     <row r="40">
@@ -34248,7 +34248,7 @@
         <v>-15.65</v>
       </c>
       <c r="C40" t="n">
-        <v>-15.2394</v>
+        <v>-15.6989</v>
       </c>
     </row>
     <row r="41">
@@ -34259,7 +34259,7 @@
         <v>15.65</v>
       </c>
       <c r="C41" t="n">
-        <v>-11.1207</v>
+        <v>-14.7799</v>
       </c>
     </row>
     <row r="42">
@@ -34270,7 +34270,7 @@
         <v>15.65</v>
       </c>
       <c r="C42" t="n">
-        <v>-2.1059</v>
+        <v>-7.4616</v>
       </c>
     </row>
     <row r="43">
@@ -34281,7 +34281,7 @@
         <v>15.65</v>
       </c>
       <c r="C43" t="n">
-        <v>6.4684</v>
+        <v>3.2498</v>
       </c>
     </row>
     <row r="44">
@@ -34292,7 +34292,7 @@
         <v>15.65</v>
       </c>
       <c r="C44" t="n">
-        <v>7.3967</v>
+        <v>9.6869</v>
       </c>
     </row>
     <row r="45">
@@ -34303,7 +34303,7 @@
         <v>-15.65</v>
       </c>
       <c r="C45" t="n">
-        <v>0.4443</v>
+        <v>5.1065</v>
       </c>
     </row>
     <row r="46">
@@ -34314,7 +34314,7 @@
         <v>-15.65</v>
       </c>
       <c r="C46" t="n">
-        <v>-6.8286</v>
+        <v>-4.218</v>
       </c>
     </row>
     <row r="47">
@@ -34325,7 +34325,7 @@
         <v>-15.65</v>
       </c>
       <c r="C47" t="n">
-        <v>-12.0507</v>
+        <v>-9.4392</v>
       </c>
     </row>
     <row r="48">
@@ -34336,7 +34336,7 @@
         <v>-15.65</v>
       </c>
       <c r="C48" t="n">
-        <v>-14.6627</v>
+        <v>-14.6622</v>
       </c>
     </row>
     <row r="49">
@@ -34347,7 +34347,7 @@
         <v>-15.65</v>
       </c>
       <c r="C49" t="n">
-        <v>-15.1634</v>
+        <v>-14.6632</v>
       </c>
     </row>
     <row r="50">
@@ -34358,7 +34358,7 @@
         <v>-15.65</v>
       </c>
       <c r="C50" t="n">
-        <v>-15.1924</v>
+        <v>-15.6637</v>
       </c>
     </row>
     <row r="51">
@@ -34369,7 +34369,7 @@
         <v>-15.65</v>
       </c>
       <c r="C51" t="n">
-        <v>-15.1143</v>
+        <v>-14.7211</v>
       </c>
     </row>
     <row r="52">
@@ -34380,7 +34380,7 @@
         <v>-15.65</v>
       </c>
       <c r="C52" t="n">
-        <v>-15.8175</v>
+        <v>-15.5075</v>
       </c>
     </row>
     <row r="53">
@@ -34391,7 +34391,7 @@
         <v>-15.65</v>
       </c>
       <c r="C53" t="n">
-        <v>-15.8453</v>
+        <v>-16.1274</v>
       </c>
     </row>
     <row r="54">
@@ -34402,7 +34402,7 @@
         <v>-15.65</v>
       </c>
       <c r="C54" t="n">
-        <v>-15.7496</v>
+        <v>-15.5632</v>
       </c>
     </row>
     <row r="55">
@@ -34413,7 +34413,7 @@
         <v>-15.65</v>
       </c>
       <c r="C55" t="n">
-        <v>-15.3755</v>
+        <v>-15.9359</v>
       </c>
     </row>
     <row r="56">
@@ -34424,7 +34424,7 @@
         <v>-15.65</v>
       </c>
       <c r="C56" t="n">
-        <v>-15.3251</v>
+        <v>-14.8151</v>
       </c>
     </row>
     <row r="57">
@@ -34435,7 +34435,7 @@
         <v>-15.65</v>
       </c>
       <c r="C57" t="n">
-        <v>-16.4004</v>
+        <v>-15.8351</v>
       </c>
     </row>
     <row r="58">
@@ -34446,7 +34446,7 @@
         <v>-15.65</v>
       </c>
       <c r="C58" t="n">
-        <v>-15.8084</v>
+        <v>-16.9657</v>
       </c>
     </row>
     <row r="59">
@@ -34457,7 +34457,7 @@
         <v>-15.65</v>
       </c>
       <c r="C59" t="n">
-        <v>-13.3588</v>
+        <v>-14.6511</v>
       </c>
     </row>
     <row r="60">
@@ -34468,7 +34468,7 @@
         <v>15.65</v>
       </c>
       <c r="C60" t="n">
-        <v>-6.4733</v>
+        <v>-12.0665</v>
       </c>
     </row>
     <row r="61">
@@ -34479,7 +34479,7 @@
         <v>15.65</v>
       </c>
       <c r="C61" t="n">
-        <v>4.5383</v>
+        <v>-0.8801</v>
       </c>
     </row>
     <row r="62">
@@ -34490,7 +34490,7 @@
         <v>15.65</v>
       </c>
       <c r="C62" t="n">
-        <v>10.5283</v>
+        <v>9.9566</v>
       </c>
     </row>
     <row r="63">
@@ -34501,7 +34501,7 @@
         <v>15.65</v>
       </c>
       <c r="C63" t="n">
-        <v>12.618</v>
+        <v>11.0999</v>
       </c>
     </row>
     <row r="64">
@@ -34512,7 +34512,7 @@
         <v>15.65</v>
       </c>
       <c r="C64" t="n">
-        <v>14.8038</v>
+        <v>14.1361</v>
       </c>
     </row>
     <row r="65">
@@ -34523,7 +34523,7 @@
         <v>15.65</v>
       </c>
       <c r="C65" t="n">
-        <v>14.2917</v>
+        <v>15.4715</v>
       </c>
     </row>
     <row r="66">
@@ -34534,7 +34534,7 @@
         <v>-15.65</v>
       </c>
       <c r="C66" t="n">
-        <v>8.9407</v>
+        <v>13.1119</v>
       </c>
     </row>
     <row r="67">
@@ -34545,7 +34545,7 @@
         <v>-15.65</v>
       </c>
       <c r="C67" t="n">
-        <v>-0.7438</v>
+        <v>4.7695</v>
       </c>
     </row>
     <row r="68">
@@ -34556,7 +34556,7 @@
         <v>-15.65</v>
       </c>
       <c r="C68" t="n">
-        <v>-8.9595</v>
+        <v>-6.257</v>
       </c>
     </row>
     <row r="69">
@@ -34567,7 +34567,7 @@
         <v>-15.65</v>
       </c>
       <c r="C69" t="n">
-        <v>-12.8721</v>
+        <v>-11.6619</v>
       </c>
     </row>
     <row r="70">
@@ -34578,7 +34578,7 @@
         <v>-15.65</v>
       </c>
       <c r="C70" t="n">
-        <v>-14.1455</v>
+        <v>-14.0823</v>
       </c>
     </row>
     <row r="71">
@@ -34589,7 +34589,7 @@
         <v>-15.65</v>
       </c>
       <c r="C71" t="n">
-        <v>-14.8365</v>
+        <v>-14.2087</v>
       </c>
     </row>
     <row r="72">
@@ -34600,7 +34600,7 @@
         <v>-15.65</v>
       </c>
       <c r="C72" t="n">
-        <v>-15.6891</v>
+        <v>-15.4643</v>
       </c>
     </row>
     <row r="73">
@@ -34611,7 +34611,7 @@
         <v>-15.65</v>
       </c>
       <c r="C73" t="n">
-        <v>-15.9257</v>
+        <v>-15.9139</v>
       </c>
     </row>
     <row r="74">
@@ -34622,7 +34622,7 @@
         <v>-15.65</v>
       </c>
       <c r="C74" t="n">
-        <v>-15.4361</v>
+        <v>-15.9375</v>
       </c>
     </row>
     <row r="75">
@@ -34633,7 +34633,7 @@
         <v>-15.65</v>
       </c>
       <c r="C75" t="n">
-        <v>-15.2521</v>
+        <v>-14.9347</v>
       </c>
     </row>
     <row r="76">
@@ -34644,7 +34644,7 @@
         <v>-15.65</v>
       </c>
       <c r="C76" t="n">
-        <v>-15.6459</v>
+        <v>-15.5696</v>
       </c>
     </row>
     <row r="77">
@@ -34655,7 +34655,7 @@
         <v>-15.65</v>
       </c>
       <c r="C77" t="n">
-        <v>-14.8322</v>
+        <v>-15.7221</v>
       </c>
     </row>
     <row r="78">
@@ -34666,7 +34666,7 @@
         <v>15.65</v>
       </c>
       <c r="C78" t="n">
-        <v>-10.2295</v>
+        <v>-13.9424</v>
       </c>
     </row>
     <row r="79">
@@ -34677,7 +34677,7 @@
         <v>15.65</v>
       </c>
       <c r="C79" t="n">
-        <v>-0.6394</v>
+        <v>-6.5167</v>
       </c>
     </row>
     <row r="80">
@@ -34688,7 +34688,7 @@
         <v>15.65</v>
       </c>
       <c r="C80" t="n">
-        <v>7.8172</v>
+        <v>5.2379</v>
       </c>
     </row>
     <row r="81">
@@ -34699,7 +34699,7 @@
         <v>-15.65</v>
       </c>
       <c r="C81" t="n">
-        <v>7.0381</v>
+        <v>10.3965</v>
       </c>
     </row>
     <row r="82">
@@ -34710,7 +34710,7 @@
         <v>-15.65</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.5802</v>
+        <v>3.6797</v>
       </c>
     </row>
     <row r="83">
@@ -34721,7 +34721,7 @@
         <v>-15.65</v>
       </c>
       <c r="C83" t="n">
-        <v>-7.9723</v>
+        <v>-4.8402</v>
       </c>
     </row>
     <row r="84">
@@ -34732,7 +34732,7 @@
         <v>15.65</v>
       </c>
       <c r="C84" t="n">
-        <v>-8.2037</v>
+        <v>-11.1044</v>
       </c>
     </row>
     <row r="85">
@@ -34743,7 +34743,7 @@
         <v>15.65</v>
       </c>
       <c r="C85" t="n">
-        <v>-0.1413</v>
+        <v>-5.3031</v>
       </c>
     </row>
     <row r="86">
@@ -34754,7 +34754,7 @@
         <v>15.65</v>
       </c>
       <c r="C86" t="n">
-        <v>7.6161</v>
+        <v>5.0205</v>
       </c>
     </row>
     <row r="87">
@@ -34765,7 +34765,7 @@
         <v>-15.65</v>
       </c>
       <c r="C87" t="n">
-        <v>10.0934</v>
+        <v>10.2117</v>
       </c>
     </row>
     <row r="88">
@@ -34776,7 +34776,7 @@
         <v>-15.65</v>
       </c>
       <c r="C88" t="n">
-        <v>5.262</v>
+        <v>9.975099999999999</v>
       </c>
     </row>
     <row r="89">
@@ -34787,7 +34787,7 @@
         <v>-15.65</v>
       </c>
       <c r="C89" t="n">
-        <v>-3.7252</v>
+        <v>0.5489000000000001</v>
       </c>
     </row>
     <row r="90">
@@ -34798,7 +34798,7 @@
         <v>-15.65</v>
       </c>
       <c r="C90" t="n">
-        <v>-10.1609</v>
+        <v>-7.9993</v>
       </c>
     </row>
     <row r="91">
@@ -34809,7 +34809,7 @@
         <v>-15.65</v>
       </c>
       <c r="C91" t="n">
-        <v>-13.8367</v>
+        <v>-12.3224</v>
       </c>
     </row>
     <row r="92">
@@ -34820,7 +34820,7 @@
         <v>-15.65</v>
       </c>
       <c r="C92" t="n">
-        <v>-15.0664</v>
+        <v>-15.3511</v>
       </c>
     </row>
     <row r="93">
@@ -34831,7 +34831,7 @@
         <v>-15.65</v>
       </c>
       <c r="C93" t="n">
-        <v>-15.3028</v>
+        <v>-14.7817</v>
       </c>
     </row>
     <row r="94">
@@ -34842,7 +34842,7 @@
         <v>-15.65</v>
       </c>
       <c r="C94" t="n">
-        <v>-15.8812</v>
+        <v>-15.8239</v>
       </c>
     </row>
     <row r="95">
@@ -34853,7 +34853,7 @@
         <v>-15.65</v>
       </c>
       <c r="C95" t="n">
-        <v>-15.8487</v>
+        <v>-15.9384</v>
       </c>
     </row>
     <row r="96">
@@ -34864,7 +34864,7 @@
         <v>-15.65</v>
       </c>
       <c r="C96" t="n">
-        <v>-12.5153</v>
+        <v>-15.7591</v>
       </c>
     </row>
     <row r="97">
@@ -34875,7 +34875,7 @@
         <v>15.65</v>
       </c>
       <c r="C97" t="n">
-        <v>-4.6509</v>
+        <v>-9.2715</v>
       </c>
     </row>
     <row r="98">
@@ -34886,7 +34886,7 @@
         <v>15.65</v>
       </c>
       <c r="C98" t="n">
-        <v>4.3191</v>
+        <v>-0.0303</v>
       </c>
     </row>
     <row r="99">
@@ -34897,7 +34897,7 @@
         <v>15.65</v>
       </c>
       <c r="C99" t="n">
-        <v>11.086</v>
+        <v>8.6685</v>
       </c>
     </row>
     <row r="100">
@@ -34908,7 +34908,7 @@
         <v>15.65</v>
       </c>
       <c r="C100" t="n">
-        <v>14.0397</v>
+        <v>13.5034</v>
       </c>
     </row>
     <row r="101">
@@ -34919,7 +34919,7 @@
         <v>15.65</v>
       </c>
       <c r="C101" t="n">
-        <v>14.6624</v>
+        <v>14.5759</v>
       </c>
     </row>
     <row r="102">
@@ -34930,7 +34930,7 @@
         <v>15.65</v>
       </c>
       <c r="C102" t="n">
-        <v>14.686</v>
+        <v>14.7489</v>
       </c>
     </row>
     <row r="103">
@@ -34941,7 +34941,7 @@
         <v>15.65</v>
       </c>
       <c r="C103" t="n">
-        <v>15.1341</v>
+        <v>14.623</v>
       </c>
     </row>
     <row r="104">
@@ -34952,7 +34952,7 @@
         <v>15.65</v>
       </c>
       <c r="C104" t="n">
-        <v>16.4005</v>
+        <v>15.6452</v>
       </c>
     </row>
     <row r="105">
@@ -34963,7 +34963,7 @@
         <v>15.65</v>
       </c>
       <c r="C105" t="n">
-        <v>15.9834</v>
+        <v>17.1557</v>
       </c>
     </row>
     <row r="106">
@@ -34974,7 +34974,7 @@
         <v>15.65</v>
       </c>
       <c r="C106" t="n">
-        <v>15.226</v>
+        <v>14.8111</v>
       </c>
     </row>
     <row r="107">
@@ -34985,7 +34985,7 @@
         <v>15.65</v>
       </c>
       <c r="C107" t="n">
-        <v>15.6944</v>
+        <v>15.6409</v>
       </c>
     </row>
     <row r="108">
@@ -34996,7 +34996,7 @@
         <v>15.65</v>
       </c>
       <c r="C108" t="n">
-        <v>14.9236</v>
+        <v>15.748</v>
       </c>
     </row>
     <row r="109">
@@ -35007,7 +35007,7 @@
         <v>-15.65</v>
       </c>
       <c r="C109" t="n">
-        <v>8.9025</v>
+        <v>14.0991</v>
       </c>
     </row>
     <row r="110">
@@ -35018,7 +35018,7 @@
         <v>-15.65</v>
       </c>
       <c r="C110" t="n">
-        <v>-2.3762</v>
+        <v>3.7059</v>
       </c>
     </row>
     <row r="111">
@@ -35029,7 +35029,7 @@
         <v>-15.65</v>
       </c>
       <c r="C111" t="n">
-        <v>-8.8565</v>
+        <v>-8.4582</v>
       </c>
     </row>
     <row r="112">
@@ -35040,7 +35040,7 @@
         <v>-15.65</v>
       </c>
       <c r="C112" t="n">
-        <v>-11.2802</v>
+        <v>-9.2547</v>
       </c>
     </row>
     <row r="113">
@@ -35051,7 +35051,7 @@
         <v>-15.65</v>
       </c>
       <c r="C113" t="n">
-        <v>-14.5778</v>
+        <v>-13.3057</v>
       </c>
     </row>
     <row r="114">
@@ -35062,7 +35062,7 @@
         <v>-15.65</v>
       </c>
       <c r="C114" t="n">
-        <v>-15.423</v>
+        <v>-15.8499</v>
       </c>
     </row>
     <row r="115">
@@ -35073,7 +35073,7 @@
         <v>15.65</v>
       </c>
       <c r="C115" t="n">
-        <v>-10.6816</v>
+        <v>-14.9962</v>
       </c>
     </row>
     <row r="116">
@@ -35084,7 +35084,7 @@
         <v>15.65</v>
       </c>
       <c r="C116" t="n">
-        <v>-1.2311</v>
+        <v>-6.3669</v>
       </c>
     </row>
     <row r="117">
@@ -35095,7 +35095,7 @@
         <v>15.65</v>
       </c>
       <c r="C117" t="n">
-        <v>7.3678</v>
+        <v>3.9048</v>
       </c>
     </row>
     <row r="118">
@@ -35106,7 +35106,7 @@
         <v>-15.65</v>
       </c>
       <c r="C118" t="n">
-        <v>7.6186</v>
+        <v>10.8308</v>
       </c>
     </row>
     <row r="119">
@@ -35117,7 +35117,7 @@
         <v>-15.65</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.4581</v>
+        <v>4.4065</v>
       </c>
     </row>
     <row r="120">
@@ -35128,7 +35128,7 @@
         <v>-15.65</v>
       </c>
       <c r="C120" t="n">
-        <v>-8.8851</v>
+        <v>-5.3227</v>
       </c>
     </row>
     <row r="121">
@@ -35139,7 +35139,7 @@
         <v>-15.65</v>
       </c>
       <c r="C121" t="n">
-        <v>-13.0798</v>
+        <v>-12.4476</v>
       </c>
     </row>
     <row r="122">
@@ -35150,7 +35150,7 @@
         <v>-15.65</v>
       </c>
       <c r="C122" t="n">
-        <v>-13.3676</v>
+        <v>-13.712</v>
       </c>
     </row>
     <row r="123">
@@ -35161,7 +35161,7 @@
         <v>-15.65</v>
       </c>
       <c r="C123" t="n">
-        <v>-14.6279</v>
+        <v>-13.0231</v>
       </c>
     </row>
     <row r="124">
@@ -35172,7 +35172,7 @@
         <v>-15.65</v>
       </c>
       <c r="C124" t="n">
-        <v>-15.5514</v>
+        <v>-16.2328</v>
       </c>
     </row>
     <row r="125">
@@ -35183,7 +35183,7 @@
         <v>-15.65</v>
       </c>
       <c r="C125" t="n">
-        <v>-16.0036</v>
+        <v>-14.8699</v>
       </c>
     </row>
     <row r="126">
@@ -35194,7 +35194,7 @@
         <v>15.65</v>
       </c>
       <c r="C126" t="n">
-        <v>-16.0522</v>
+        <v>-17.1372</v>
       </c>
     </row>
     <row r="127">
@@ -35205,7 +35205,7 @@
         <v>15.65</v>
       </c>
       <c r="C127" t="n">
-        <v>-12.7452</v>
+        <v>-14.9673</v>
       </c>
     </row>
     <row r="128">
@@ -35216,7 +35216,7 @@
         <v>15.65</v>
       </c>
       <c r="C128" t="n">
-        <v>-5.0379</v>
+        <v>-10.5232</v>
       </c>
     </row>
     <row r="129">
@@ -35227,7 +35227,7 @@
         <v>15.65</v>
       </c>
       <c r="C129" t="n">
-        <v>4.3371</v>
+        <v>0.4475</v>
       </c>
     </row>
     <row r="130">
@@ -35238,7 +35238,7 @@
         <v>-15.65</v>
       </c>
       <c r="C130" t="n">
-        <v>9.535600000000001</v>
+        <v>8.226699999999999</v>
       </c>
     </row>
     <row r="131">
@@ -35249,7 +35249,7 @@
         <v>-15.65</v>
       </c>
       <c r="C131" t="n">
-        <v>4.9705</v>
+        <v>10.8444</v>
       </c>
     </row>
     <row r="132">
@@ -35260,7 +35260,7 @@
         <v>-15.65</v>
       </c>
       <c r="C132" t="n">
-        <v>-4.3076</v>
+        <v>-0.9033</v>
       </c>
     </row>
     <row r="133">
@@ -35271,7 +35271,7 @@
         <v>15.65</v>
       </c>
       <c r="C133" t="n">
-        <v>-5.4546</v>
+        <v>-7.7119</v>
       </c>
     </row>
     <row r="134">
@@ -35282,7 +35282,7 @@
         <v>15.65</v>
       </c>
       <c r="C134" t="n">
-        <v>1.0509</v>
+        <v>-3.1973</v>
       </c>
     </row>
     <row r="135">
@@ -35293,7 +35293,7 @@
         <v>15.65</v>
       </c>
       <c r="C135" t="n">
-        <v>8.865</v>
+        <v>5.2992</v>
       </c>
     </row>
     <row r="136">
@@ -35304,7 +35304,7 @@
         <v>15.65</v>
       </c>
       <c r="C136" t="n">
-        <v>12.748</v>
+        <v>12.4307</v>
       </c>
     </row>
     <row r="137">
@@ -35315,7 +35315,7 @@
         <v>15.65</v>
       </c>
       <c r="C137" t="n">
-        <v>14.0483</v>
+        <v>13.0653</v>
       </c>
     </row>
     <row r="138">
@@ -35326,7 +35326,7 @@
         <v>15.65</v>
       </c>
       <c r="C138" t="n">
-        <v>14.3639</v>
+        <v>15.0313</v>
       </c>
     </row>
     <row r="139">
@@ -35337,7 +35337,7 @@
         <v>-15.65</v>
       </c>
       <c r="C139" t="n">
-        <v>7.2573</v>
+        <v>13.6966</v>
       </c>
     </row>
     <row r="140">
@@ -35348,7 +35348,7 @@
         <v>-15.65</v>
       </c>
       <c r="C140" t="n">
-        <v>0.1475</v>
+        <v>0.8179</v>
       </c>
     </row>
     <row r="141">
@@ -35359,7 +35359,7 @@
         <v>-15.65</v>
       </c>
       <c r="C141" t="n">
-        <v>-5.8894</v>
+        <v>-0.523</v>
       </c>
     </row>
     <row r="142">
@@ -35370,7 +35370,7 @@
         <v>-15.65</v>
       </c>
       <c r="C142" t="n">
-        <v>-12.5398</v>
+        <v>-11.2558</v>
       </c>
     </row>
     <row r="143">
@@ -35381,7 +35381,7 @@
         <v>-15.65</v>
       </c>
       <c r="C143" t="n">
-        <v>-14.351</v>
+        <v>-13.8239</v>
       </c>
     </row>
     <row r="144">
@@ -35392,7 +35392,7 @@
         <v>-15.65</v>
       </c>
       <c r="C144" t="n">
-        <v>-15.406</v>
+        <v>-14.8782</v>
       </c>
     </row>
     <row r="145">
@@ -35403,7 +35403,7 @@
         <v>-15.65</v>
       </c>
       <c r="C145" t="n">
-        <v>-12.4081</v>
+        <v>-15.9338</v>
       </c>
     </row>
     <row r="146">
@@ -35414,7 +35414,7 @@
         <v>15.65</v>
       </c>
       <c r="C146" t="n">
-        <v>-3.1431</v>
+        <v>-8.882400000000001</v>
       </c>
     </row>
     <row r="147">
@@ -35425,7 +35425,7 @@
         <v>15.65</v>
       </c>
       <c r="C147" t="n">
-        <v>5.8957</v>
+        <v>2.5963</v>
       </c>
     </row>
     <row r="148">
@@ -35436,7 +35436,7 @@
         <v>15.65</v>
       </c>
       <c r="C148" t="n">
-        <v>10.9534</v>
+        <v>9.1952</v>
       </c>
     </row>
     <row r="149">
@@ -35447,7 +35447,7 @@
         <v>15.65</v>
       </c>
       <c r="C149" t="n">
-        <v>14.4481</v>
+        <v>12.7116</v>
       </c>
     </row>
     <row r="150">
@@ -35458,7 +35458,7 @@
         <v>15.65</v>
       </c>
       <c r="C150" t="n">
-        <v>15.457</v>
+        <v>16.1847</v>
       </c>
     </row>
     <row r="151">
@@ -35469,7 +35469,7 @@
         <v>15.65</v>
       </c>
       <c r="C151" t="n">
-        <v>14.731</v>
+        <v>14.7293</v>
       </c>
     </row>
     <row r="152">
@@ -35480,7 +35480,7 @@
         <v>15.65</v>
       </c>
       <c r="C152" t="n">
-        <v>15.3977</v>
+        <v>14.7327</v>
       </c>
     </row>
     <row r="153">
@@ -35491,7 +35491,7 @@
         <v>15.65</v>
       </c>
       <c r="C153" t="n">
-        <v>15.5566</v>
+        <v>16.0628</v>
       </c>
     </row>
     <row r="154">
@@ -35502,7 +35502,7 @@
         <v>15.65</v>
       </c>
       <c r="C154" t="n">
-        <v>12.7441</v>
+        <v>15.0503</v>
       </c>
     </row>
     <row r="155">
@@ -35513,7 +35513,7 @@
         <v>-15.65</v>
       </c>
       <c r="C155" t="n">
-        <v>3.7991</v>
+        <v>10.4379</v>
       </c>
     </row>
     <row r="156">
@@ -35524,7 +35524,7 @@
         <v>-15.65</v>
       </c>
       <c r="C156" t="n">
-        <v>-6.1374</v>
+        <v>-2.8396</v>
       </c>
     </row>
     <row r="157">
@@ -35535,7 +35535,7 @@
         <v>-15.65</v>
       </c>
       <c r="C157" t="n">
-        <v>-10.1408</v>
+        <v>-9.4351</v>
       </c>
     </row>
     <row r="158">
@@ -35546,7 +35546,7 @@
         <v>15.65</v>
       </c>
       <c r="C158" t="n">
-        <v>-5.8161</v>
+        <v>-10.8466</v>
       </c>
     </row>
     <row r="159">
@@ -35557,7 +35557,7 @@
         <v>15.65</v>
       </c>
       <c r="C159" t="n">
-        <v>3.5211</v>
+        <v>-0.7857</v>
       </c>
     </row>
     <row r="160">
@@ -35568,7 +35568,7 @@
         <v>15.65</v>
       </c>
       <c r="C160" t="n">
-        <v>7.1267</v>
+        <v>7.8278</v>
       </c>
     </row>
     <row r="161">
@@ -35579,7 +35579,7 @@
         <v>-15.65</v>
       </c>
       <c r="C161" t="n">
-        <v>2.6865</v>
+        <v>6.4257</v>
       </c>
     </row>
     <row r="162">
@@ -35590,7 +35590,7 @@
         <v>-15.65</v>
       </c>
       <c r="C162" t="n">
-        <v>-5.1098</v>
+        <v>-1.0527</v>
       </c>
     </row>
     <row r="163">
@@ -35601,7 +35601,7 @@
         <v>-15.65</v>
       </c>
       <c r="C163" t="n">
-        <v>-10.101</v>
+        <v>-9.1668</v>
       </c>
     </row>
     <row r="164">
@@ -35612,7 +35612,7 @@
         <v>15.65</v>
       </c>
       <c r="C164" t="n">
-        <v>-5.5287</v>
+        <v>-11.0351</v>
       </c>
     </row>
     <row r="165">
@@ -35623,7 +35623,7 @@
         <v>15.65</v>
       </c>
       <c r="C165" t="n">
-        <v>3.5796</v>
+        <v>-0.0223</v>
       </c>
     </row>
     <row r="166">
@@ -35634,7 +35634,7 @@
         <v>15.65</v>
       </c>
       <c r="C166" t="n">
-        <v>8.388</v>
+        <v>7.1816</v>
       </c>
     </row>
     <row r="167">
@@ -35645,7 +35645,7 @@
         <v>-15.65</v>
       </c>
       <c r="C167" t="n">
-        <v>5.9069</v>
+        <v>9.5943</v>
       </c>
     </row>
     <row r="168">
@@ -35656,7 +35656,7 @@
         <v>-15.65</v>
       </c>
       <c r="C168" t="n">
-        <v>-3.9377</v>
+        <v>2.2195</v>
       </c>
     </row>
     <row r="169">
@@ -35667,7 +35667,7 @@
         <v>-15.65</v>
       </c>
       <c r="C169" t="n">
-        <v>-10.1175</v>
+        <v>-10.0949</v>
       </c>
     </row>
     <row r="170">
@@ -35678,7 +35678,7 @@
         <v>-15.65</v>
       </c>
       <c r="C170" t="n">
-        <v>-12.1209</v>
+        <v>-10.14</v>
       </c>
     </row>
     <row r="171">
@@ -35689,7 +35689,7 @@
         <v>-15.65</v>
       </c>
       <c r="C171" t="n">
-        <v>-14.5984</v>
+        <v>-14.1018</v>
       </c>
     </row>
     <row r="172">
@@ -35700,7 +35700,7 @@
         <v>-15.65</v>
       </c>
       <c r="C172" t="n">
-        <v>-11.8169</v>
+        <v>-15.0949</v>
       </c>
     </row>
     <row r="173">
@@ -35711,7 +35711,7 @@
         <v>15.65</v>
       </c>
       <c r="C173" t="n">
-        <v>-8.157500000000001</v>
+        <v>-8.5389</v>
       </c>
     </row>
     <row r="174">
@@ -35722,7 +35722,7 @@
         <v>15.65</v>
       </c>
       <c r="C174" t="n">
-        <v>-0.2532</v>
+        <v>-7.776</v>
       </c>
     </row>
     <row r="175">
@@ -35733,7 +35733,7 @@
         <v>15.65</v>
       </c>
       <c r="C175" t="n">
-        <v>9.230499999999999</v>
+        <v>7.2696</v>
       </c>
     </row>
     <row r="176">
@@ -35744,7 +35744,7 @@
         <v>15.65</v>
       </c>
       <c r="C176" t="n">
-        <v>13.0136</v>
+        <v>11.1914</v>
       </c>
     </row>
     <row r="177">
@@ -35755,7 +35755,7 @@
         <v>15.65</v>
       </c>
       <c r="C177" t="n">
-        <v>15.0535</v>
+        <v>14.8358</v>
       </c>
     </row>
     <row r="178">
@@ -35766,7 +35766,7 @@
         <v>15.65</v>
       </c>
       <c r="C178" t="n">
-        <v>15.4234</v>
+        <v>15.2712</v>
       </c>
     </row>
     <row r="179">
@@ -35777,7 +35777,7 @@
         <v>15.65</v>
       </c>
       <c r="C179" t="n">
-        <v>15.144</v>
+        <v>15.5757</v>
       </c>
     </row>
     <row r="180">
@@ -35788,7 +35788,7 @@
         <v>15.65</v>
       </c>
       <c r="C180" t="n">
-        <v>15.0478</v>
+        <v>14.7123</v>
       </c>
     </row>
     <row r="181">
@@ -35799,7 +35799,7 @@
         <v>15.65</v>
       </c>
       <c r="C181" t="n">
-        <v>14.94</v>
+        <v>15.3832</v>
       </c>
     </row>
     <row r="182">
@@ -35810,7 +35810,7 @@
         <v>15.65</v>
       </c>
       <c r="C182" t="n">
-        <v>16.1279</v>
+        <v>14.4967</v>
       </c>
     </row>
     <row r="183">
@@ -35821,7 +35821,7 @@
         <v>15.65</v>
       </c>
       <c r="C183" t="n">
-        <v>16.7183</v>
+        <v>17.7591</v>
       </c>
     </row>
     <row r="184">
@@ -35832,7 +35832,7 @@
         <v>15.65</v>
       </c>
       <c r="C184" t="n">
-        <v>15.209</v>
+        <v>15.6776</v>
       </c>
     </row>
     <row r="185">
@@ -35843,7 +35843,7 @@
         <v>15.65</v>
       </c>
       <c r="C185" t="n">
-        <v>14.7295</v>
+        <v>14.7405</v>
       </c>
     </row>
     <row r="186">
@@ -35854,7 +35854,7 @@
         <v>15.65</v>
       </c>
       <c r="C186" t="n">
-        <v>15.0871</v>
+        <v>14.7186</v>
       </c>
     </row>
     <row r="187">
@@ -35865,7 +35865,7 @@
         <v>15.65</v>
       </c>
       <c r="C187" t="n">
-        <v>16.4792</v>
+        <v>15.4555</v>
       </c>
     </row>
     <row r="188">
@@ -35876,7 +35876,7 @@
         <v>-15.65</v>
       </c>
       <c r="C188" t="n">
-        <v>12.2359</v>
+        <v>17.503</v>
       </c>
     </row>
     <row r="189">
@@ -35887,7 +35887,7 @@
         <v>-15.65</v>
       </c>
       <c r="C189" t="n">
-        <v>1.6858</v>
+        <v>6.9688</v>
       </c>
     </row>
     <row r="190">
@@ -35898,7 +35898,7 @@
         <v>-15.65</v>
       </c>
       <c r="C190" t="n">
-        <v>-6.9998</v>
+        <v>-3.5971</v>
       </c>
     </row>
     <row r="191">
@@ -35909,7 +35909,7 @@
         <v>15.65</v>
       </c>
       <c r="C191" t="n">
-        <v>-8.6197</v>
+        <v>-10.4025</v>
       </c>
     </row>
     <row r="192">
@@ -35920,7 +35920,7 @@
         <v>15.65</v>
       </c>
       <c r="C192" t="n">
-        <v>-1.9203</v>
+        <v>-6.8369</v>
       </c>
     </row>
     <row r="193">
@@ -35931,7 +35931,7 @@
         <v>15.65</v>
       </c>
       <c r="C193" t="n">
-        <v>6.3916</v>
+        <v>2.9962</v>
       </c>
     </row>
     <row r="194">
@@ -35942,7 +35942,7 @@
         <v>15.65</v>
       </c>
       <c r="C194" t="n">
-        <v>9.321999999999999</v>
+        <v>9.787100000000001</v>
       </c>
     </row>
     <row r="195">
@@ -35953,7 +35953,7 @@
         <v>-15.65</v>
       </c>
       <c r="C195" t="n">
-        <v>3.6883</v>
+        <v>8.856999999999999</v>
       </c>
     </row>
     <row r="196">
@@ -35964,7 +35964,7 @@
         <v>-15.65</v>
       </c>
       <c r="C196" t="n">
-        <v>-4.7853</v>
+        <v>-1.4804</v>
       </c>
     </row>
     <row r="197">
@@ -35975,7 +35975,7 @@
         <v>-15.65</v>
       </c>
       <c r="C197" t="n">
-        <v>-10.9995</v>
+        <v>-8.090199999999999</v>
       </c>
     </row>
     <row r="198">
@@ -35986,7 +35986,7 @@
         <v>-15.65</v>
       </c>
       <c r="C198" t="n">
-        <v>-13.8014</v>
+        <v>-13.9089</v>
       </c>
     </row>
     <row r="199">
@@ -35997,7 +35997,7 @@
         <v>-15.65</v>
       </c>
       <c r="C199" t="n">
-        <v>-14.688</v>
+        <v>-13.694</v>
       </c>
     </row>
     <row r="200">
@@ -36008,7 +36008,7 @@
         <v>-15.65</v>
       </c>
       <c r="C200" t="n">
-        <v>-15.219</v>
+        <v>-15.682</v>
       </c>
     </row>
     <row r="201">
@@ -36019,7 +36019,7 @@
         <v>-15.65</v>
       </c>
       <c r="C201" t="n">
-        <v>-14.7372</v>
+        <v>-14.7559</v>
       </c>
     </row>
     <row r="202">
@@ -36030,7 +36030,7 @@
         <v>-15.65</v>
       </c>
       <c r="C202" t="n">
-        <v>-15.8864</v>
+        <v>-14.7185</v>
       </c>
     </row>
     <row r="203">
@@ -36041,7 +36041,7 @@
         <v>-15.65</v>
       </c>
       <c r="C203" t="n">
-        <v>-16.3367</v>
+        <v>-17.0542</v>
       </c>
     </row>
     <row r="204">
@@ -36052,7 +36052,7 @@
         <v>-15.65</v>
       </c>
       <c r="C204" t="n">
-        <v>-15.6361</v>
+        <v>-15.6191</v>
       </c>
     </row>
     <row r="205">
@@ -36063,7 +36063,7 @@
         <v>-15.65</v>
       </c>
       <c r="C205" t="n">
-        <v>-15.2813</v>
+        <v>-15.6532</v>
       </c>
     </row>
     <row r="206">
@@ -36074,7 +36074,7 @@
         <v>-15.65</v>
       </c>
       <c r="C206" t="n">
-        <v>-14.8852</v>
+        <v>-14.9094</v>
       </c>
     </row>
     <row r="207">
@@ -36085,7 +36085,7 @@
         <v>-15.65</v>
       </c>
       <c r="C207" t="n">
-        <v>-11.4574</v>
+        <v>-14.861</v>
       </c>
     </row>
     <row r="208">
@@ -36096,7 +36096,7 @@
         <v>15.65</v>
       </c>
       <c r="C208" t="n">
-        <v>-1.7499</v>
+        <v>-8.053800000000001</v>
       </c>
     </row>
     <row r="209">
@@ -36107,7 +36107,7 @@
         <v>15.65</v>
       </c>
       <c r="C209" t="n">
-        <v>7.9914</v>
+        <v>4.5541</v>
       </c>
     </row>
     <row r="210">
@@ -36118,7 +36118,7 @@
         <v>15.65</v>
       </c>
       <c r="C210" t="n">
-        <v>11.6638</v>
+        <v>11.4287</v>
       </c>
     </row>
     <row r="211">
@@ -36129,7 +36129,7 @@
         <v>15.65</v>
       </c>
       <c r="C211" t="n">
-        <v>13.9432</v>
+        <v>11.8989</v>
       </c>
     </row>
     <row r="212">
@@ -36140,7 +36140,7 @@
         <v>15.65</v>
       </c>
       <c r="C212" t="n">
-        <v>15.8446</v>
+        <v>15.9876</v>
       </c>
     </row>
     <row r="213">
@@ -36151,7 +36151,7 @@
         <v>15.65</v>
       </c>
       <c r="C213" t="n">
-        <v>15.2062</v>
+        <v>15.7017</v>
       </c>
     </row>
     <row r="214">
@@ -36162,7 +36162,7 @@
         <v>15.65</v>
       </c>
       <c r="C214" t="n">
-        <v>15.048</v>
+        <v>14.7107</v>
       </c>
     </row>
     <row r="215">
@@ -36173,7 +36173,7 @@
         <v>15.65</v>
       </c>
       <c r="C215" t="n">
-        <v>15.2088</v>
+        <v>15.3853</v>
       </c>
     </row>
     <row r="216">
@@ -36184,7 +36184,7 @@
         <v>-15.65</v>
       </c>
       <c r="C216" t="n">
-        <v>11.0987</v>
+        <v>15.0323</v>
       </c>
     </row>
     <row r="217">
@@ -36195,7 +36195,7 @@
         <v>-15.65</v>
       </c>
       <c r="C217" t="n">
-        <v>1.1364</v>
+        <v>7.1651</v>
       </c>
     </row>
     <row r="218">
@@ -36206,7 +36206,7 @@
         <v>-15.65</v>
       </c>
       <c r="C218" t="n">
-        <v>-8.228300000000001</v>
+        <v>-4.8924</v>
       </c>
     </row>
     <row r="219">
@@ -36217,7 +36217,7 @@
         <v>-15.65</v>
       </c>
       <c r="C219" t="n">
-        <v>-12.1607</v>
+        <v>-11.5642</v>
       </c>
     </row>
     <row r="220">
@@ -36228,7 +36228,7 @@
         <v>-15.65</v>
       </c>
       <c r="C220" t="n">
-        <v>-13.4828</v>
+        <v>-12.7573</v>
       </c>
     </row>
     <row r="221">
@@ -36239,7 +36239,7 @@
         <v>-15.65</v>
       </c>
       <c r="C221" t="n">
-        <v>-15.8817</v>
+        <v>-14.2084</v>
       </c>
     </row>
     <row r="222">
@@ -36250,7 +36250,7 @@
         <v>-15.65</v>
       </c>
       <c r="C222" t="n">
-        <v>-16.1249</v>
+        <v>-17.555</v>
       </c>
     </row>
     <row r="223">
@@ -36261,7 +36261,7 @@
         <v>-15.65</v>
       </c>
       <c r="C223" t="n">
-        <v>-15.1496</v>
+        <v>-14.6947</v>
       </c>
     </row>
     <row r="224">
@@ -36272,7 +36272,7 @@
         <v>-15.65</v>
       </c>
       <c r="C224" t="n">
-        <v>-15.1832</v>
+        <v>-15.6045</v>
       </c>
     </row>
     <row r="225">
@@ -36283,7 +36283,7 @@
         <v>15.65</v>
       </c>
       <c r="C225" t="n">
-        <v>-11.526</v>
+        <v>-14.7619</v>
       </c>
     </row>
     <row r="226">
@@ -36294,7 +36294,7 @@
         <v>15.65</v>
       </c>
       <c r="C226" t="n">
-        <v>-2.5128</v>
+        <v>-8.2902</v>
       </c>
     </row>
     <row r="227">
@@ -36305,7 +36305,7 @@
         <v>15.65</v>
       </c>
       <c r="C227" t="n">
-        <v>6.5671</v>
+        <v>3.2646</v>
       </c>
     </row>
     <row r="228">
@@ -36316,7 +36316,7 @@
         <v>-15.65</v>
       </c>
       <c r="C228" t="n">
-        <v>9.3537</v>
+        <v>9.8695</v>
       </c>
     </row>
     <row r="229">
@@ -36327,7 +36327,7 @@
         <v>-15.65</v>
       </c>
       <c r="C229" t="n">
-        <v>3.6576</v>
+        <v>8.8378</v>
       </c>
     </row>
     <row r="230">
@@ -36338,7 +36338,7 @@
         <v>-15.65</v>
       </c>
       <c r="C230" t="n">
-        <v>-5.4411</v>
+        <v>-1.5227</v>
       </c>
     </row>
     <row r="231">
@@ -36349,7 +36349,7 @@
         <v>-15.65</v>
       </c>
       <c r="C231" t="n">
-        <v>-11.36</v>
+        <v>-9.359500000000001</v>
       </c>
     </row>
     <row r="232">
@@ -36360,7 +36360,7 @@
         <v>-15.65</v>
       </c>
       <c r="C232" t="n">
-        <v>-14.0109</v>
+        <v>-13.3604</v>
       </c>
     </row>
     <row r="233">
@@ -36371,7 +36371,7 @@
         <v>-15.65</v>
       </c>
       <c r="C233" t="n">
-        <v>-14.6902</v>
+        <v>-14.6614</v>
       </c>
     </row>
     <row r="234">
@@ -36382,7 +36382,7 @@
         <v>15.65</v>
       </c>
       <c r="C234" t="n">
-        <v>-12.4265</v>
+        <v>-14.7189</v>
       </c>
     </row>
     <row r="235">
@@ -36393,7 +36393,7 @@
         <v>15.65</v>
       </c>
       <c r="C235" t="n">
-        <v>-4.5166</v>
+        <v>-10.1342</v>
       </c>
     </row>
     <row r="236">
@@ -36404,7 +36404,7 @@
         <v>15.65</v>
       </c>
       <c r="C236" t="n">
-        <v>5.2741</v>
+        <v>1.1011</v>
       </c>
     </row>
     <row r="237">
@@ -36415,7 +36415,7 @@
         <v>-15.65</v>
       </c>
       <c r="C237" t="n">
-        <v>8.795199999999999</v>
+        <v>9.447100000000001</v>
       </c>
     </row>
     <row r="238">
@@ -36426,7 +36426,7 @@
         <v>-15.65</v>
       </c>
       <c r="C238" t="n">
-        <v>3.3531</v>
+        <v>8.1434</v>
       </c>
     </row>
     <row r="239">
@@ -36437,7 +36437,7 @@
         <v>-15.65</v>
       </c>
       <c r="C239" t="n">
-        <v>-4.8939</v>
+        <v>-1.4372</v>
       </c>
     </row>
     <row r="240">
@@ -36448,7 +36448,7 @@
         <v>-15.65</v>
       </c>
       <c r="C240" t="n">
-        <v>-11.0183</v>
+        <v>-8.3505</v>
       </c>
     </row>
     <row r="241">
@@ -36459,7 +36459,7 @@
         <v>-15.65</v>
       </c>
       <c r="C241" t="n">
-        <v>-13.5571</v>
+        <v>-13.6862</v>
       </c>
     </row>
     <row r="242">
@@ -36470,7 +36470,7 @@
         <v>-15.65</v>
       </c>
       <c r="C242" t="n">
-        <v>-14.6801</v>
+        <v>-13.428</v>
       </c>
     </row>
     <row r="243">
@@ -36481,7 +36481,7 @@
         <v>15.65</v>
       </c>
       <c r="C243" t="n">
-        <v>-14.415</v>
+        <v>-15.9322</v>
       </c>
     </row>
     <row r="244">
@@ -36492,7 +36492,7 @@
         <v>15.65</v>
       </c>
       <c r="C244" t="n">
-        <v>-7.7825</v>
+        <v>-12.8978</v>
       </c>
     </row>
     <row r="245">
@@ -36503,7 +36503,7 @@
         <v>15.65</v>
       </c>
       <c r="C245" t="n">
-        <v>2.0377</v>
+        <v>-2.6672</v>
       </c>
     </row>
     <row r="246">
@@ -36514,7 +36514,7 @@
         <v>15.65</v>
       </c>
       <c r="C246" t="n">
-        <v>9.945</v>
+        <v>6.7425</v>
       </c>
     </row>
     <row r="247">
@@ -36525,7 +36525,7 @@
         <v>15.65</v>
       </c>
       <c r="C247" t="n">
-        <v>13.1785</v>
+        <v>13.1476</v>
       </c>
     </row>
     <row r="248">
@@ -36536,7 +36536,7 @@
         <v>15.65</v>
       </c>
       <c r="C248" t="n">
-        <v>13.849</v>
+        <v>13.2094</v>
       </c>
     </row>
     <row r="249">
@@ -36547,7 +36547,7 @@
         <v>15.65</v>
       </c>
       <c r="C249" t="n">
-        <v>14.8682</v>
+        <v>14.4887</v>
       </c>
     </row>
     <row r="250">
@@ -36558,7 +36558,7 @@
         <v>-15.65</v>
       </c>
       <c r="C250" t="n">
-        <v>8.606199999999999</v>
+        <v>15.2477</v>
       </c>
     </row>
     <row r="251">
@@ -36569,7 +36569,7 @@
         <v>-15.65</v>
       </c>
       <c r="C251" t="n">
-        <v>-2.3784</v>
+        <v>1.9646</v>
       </c>
     </row>
     <row r="252">
@@ -36580,7 +36580,7 @@
         <v>-15.65</v>
       </c>
       <c r="C252" t="n">
-        <v>-8.203200000000001</v>
+        <v>-6.7215</v>
       </c>
     </row>
     <row r="253">
@@ -36591,7 +36591,7 @@
         <v>15.65</v>
       </c>
       <c r="C253" t="n">
-        <v>-6.5158</v>
+        <v>-9.684900000000001</v>
       </c>
     </row>
     <row r="254">
@@ -36602,7 +36602,7 @@
         <v>15.65</v>
       </c>
       <c r="C254" t="n">
-        <v>1.7396</v>
+        <v>-3.3468</v>
       </c>
     </row>
     <row r="255">
@@ -36613,7 +36613,7 @@
         <v>15.65</v>
       </c>
       <c r="C255" t="n">
-        <v>9.3185</v>
+        <v>6.826</v>
       </c>
     </row>
     <row r="256">
@@ -36624,7 +36624,7 @@
         <v>15.65</v>
       </c>
       <c r="C256" t="n">
-        <v>12.7435</v>
+        <v>11.811</v>
       </c>
     </row>
     <row r="257">
@@ -36635,7 +36635,7 @@
         <v>15.65</v>
       </c>
       <c r="C257" t="n">
-        <v>14.1878</v>
+        <v>13.676</v>
       </c>
     </row>
     <row r="258">
@@ -36646,7 +36646,7 @@
         <v>15.65</v>
       </c>
       <c r="C258" t="n">
-        <v>14.6966</v>
+        <v>14.6995</v>
       </c>
     </row>
     <row r="259">
@@ -36657,7 +36657,7 @@
         <v>-15.65</v>
       </c>
       <c r="C259" t="n">
-        <v>11.8811</v>
+        <v>14.6937</v>
       </c>
     </row>
     <row r="260">
@@ -36668,7 +36668,7 @@
         <v>-15.65</v>
       </c>
       <c r="C260" t="n">
-        <v>2.5677</v>
+        <v>9.0685</v>
       </c>
     </row>
     <row r="261">
@@ -36679,7 +36679,7 @@
         <v>-15.65</v>
       </c>
       <c r="C261" t="n">
-        <v>-6.8216</v>
+        <v>-3.9331</v>
       </c>
     </row>
     <row r="262">
@@ -36690,7 +36690,7 @@
         <v>15.65</v>
       </c>
       <c r="C262" t="n">
-        <v>-7.3896</v>
+        <v>-9.710000000000001</v>
       </c>
     </row>
     <row r="263">
@@ -36701,7 +36701,7 @@
         <v>15.65</v>
       </c>
       <c r="C263" t="n">
-        <v>-0.3631</v>
+        <v>-5.0692</v>
       </c>
     </row>
     <row r="264">
@@ -36712,7 +36712,7 @@
         <v>15.65</v>
       </c>
       <c r="C264" t="n">
-        <v>7.6081</v>
+        <v>4.343</v>
       </c>
     </row>
     <row r="265">
@@ -36723,7 +36723,7 @@
         <v>-15.65</v>
       </c>
       <c r="C265" t="n">
-        <v>8.468400000000001</v>
+        <v>10.8733</v>
       </c>
     </row>
     <row r="266">
@@ -36734,7 +36734,7 @@
         <v>-15.65</v>
       </c>
       <c r="C266" t="n">
-        <v>1.2178</v>
+        <v>6.0635</v>
       </c>
     </row>
     <row r="267">
@@ -36745,7 +36745,7 @@
         <v>15.65</v>
       </c>
       <c r="C267" t="n">
-        <v>-7.1851</v>
+        <v>-3.628</v>
       </c>
     </row>
     <row r="268">
@@ -36756,7 +36756,7 @@
         <v>15.65</v>
       </c>
       <c r="C268" t="n">
-        <v>-10.7629</v>
+        <v>-10.7422</v>
       </c>
     </row>
     <row r="269">
@@ -36767,7 +36767,7 @@
         <v>15.65</v>
       </c>
       <c r="C269" t="n">
-        <v>-6.0682</v>
+        <v>-10.7836</v>
       </c>
     </row>
     <row r="270">
@@ -36778,7 +36778,7 @@
         <v>15.65</v>
       </c>
       <c r="C270" t="n">
-        <v>2.9928</v>
+        <v>-1.3529</v>
       </c>
     </row>
     <row r="271">
@@ -36789,7 +36789,7 @@
         <v>15.65</v>
       </c>
       <c r="C271" t="n">
-        <v>9.978400000000001</v>
+        <v>7.3386</v>
       </c>
     </row>
     <row r="272">
@@ -36800,7 +36800,7 @@
         <v>15.65</v>
       </c>
       <c r="C272" t="n">
-        <v>13.1719</v>
+        <v>12.6182</v>
       </c>
     </row>
     <row r="273">
@@ -36811,7 +36811,7 @@
         <v>15.65</v>
       </c>
       <c r="C273" t="n">
-        <v>14.1782</v>
+        <v>13.7255</v>
       </c>
     </row>
     <row r="274">
@@ -36822,7 +36822,7 @@
         <v>-15.65</v>
       </c>
       <c r="C274" t="n">
-        <v>13.2433</v>
+        <v>14.6309</v>
       </c>
     </row>
     <row r="275">
@@ -36833,7 +36833,7 @@
         <v>-15.65</v>
       </c>
       <c r="C275" t="n">
-        <v>4.4059</v>
+        <v>11.8557</v>
       </c>
     </row>
     <row r="276">
@@ -36844,7 +36844,7 @@
         <v>-15.65</v>
       </c>
       <c r="C276" t="n">
-        <v>-3.5659</v>
+        <v>-3.0439</v>
       </c>
     </row>
     <row r="277">
@@ -36855,7 +36855,7 @@
         <v>-15.65</v>
       </c>
       <c r="C277" t="n">
-        <v>-7.4537</v>
+        <v>-4.0879</v>
       </c>
     </row>
     <row r="278">
@@ -36866,7 +36866,7 @@
         <v>15.65</v>
       </c>
       <c r="C278" t="n">
-        <v>-6.502</v>
+        <v>-10.8196</v>
       </c>
     </row>
     <row r="279">
@@ -36877,7 +36877,7 @@
         <v>15.65</v>
       </c>
       <c r="C279" t="n">
-        <v>2.1235</v>
+        <v>-2.1843</v>
       </c>
     </row>
     <row r="280">
@@ -36888,7 +36888,7 @@
         <v>15.65</v>
       </c>
       <c r="C280" t="n">
-        <v>8.9579</v>
+        <v>6.4314</v>
       </c>
     </row>
     <row r="281">
@@ -36899,7 +36899,7 @@
         <v>15.65</v>
       </c>
       <c r="C281" t="n">
-        <v>13.1937</v>
+        <v>11.4844</v>
       </c>
     </row>
     <row r="282">
@@ -36910,7 +36910,7 @@
         <v>15.65</v>
       </c>
       <c r="C282" t="n">
-        <v>15.3084</v>
+        <v>14.903</v>
       </c>
     </row>
     <row r="283">
@@ -36921,7 +36921,7 @@
         <v>15.65</v>
       </c>
       <c r="C283" t="n">
-        <v>15.4467</v>
+        <v>15.7139</v>
       </c>
     </row>
     <row r="284">
@@ -36932,7 +36932,7 @@
         <v>15.65</v>
       </c>
       <c r="C284" t="n">
-        <v>15.1729</v>
+        <v>15.1796</v>
       </c>
     </row>
     <row r="285">
@@ -36943,7 +36943,7 @@
         <v>15.65</v>
       </c>
       <c r="C285" t="n">
-        <v>14.925</v>
+        <v>15.1663</v>
       </c>
     </row>
     <row r="286">
@@ -36954,7 +36954,7 @@
         <v>15.65</v>
       </c>
       <c r="C286" t="n">
-        <v>15.9285</v>
+        <v>14.6837</v>
       </c>
     </row>
     <row r="287">
@@ -36965,7 +36965,7 @@
         <v>15.65</v>
       </c>
       <c r="C287" t="n">
-        <v>15.939</v>
+        <v>17.1734</v>
       </c>
     </row>
     <row r="288">
@@ -36976,7 +36976,7 @@
         <v>15.65</v>
       </c>
       <c r="C288" t="n">
-        <v>15.1868</v>
+        <v>14.7046</v>
       </c>
     </row>
     <row r="289">
@@ -36987,7 +36987,7 @@
         <v>15.65</v>
       </c>
       <c r="C289" t="n">
-        <v>14.7348</v>
+        <v>15.6689</v>
       </c>
     </row>
     <row r="290">
@@ -36998,7 +36998,7 @@
         <v>-15.65</v>
       </c>
       <c r="C290" t="n">
-        <v>9.3828</v>
+        <v>13.8008</v>
       </c>
     </row>
     <row r="291">
@@ -37009,7 +37009,7 @@
         <v>-15.65</v>
       </c>
       <c r="C291" t="n">
-        <v>-0.4559</v>
+        <v>4.9647</v>
       </c>
     </row>
     <row r="292">
@@ -37020,7 +37020,7 @@
         <v>-15.65</v>
       </c>
       <c r="C292" t="n">
-        <v>-8.2989</v>
+        <v>-5.8766</v>
       </c>
     </row>
     <row r="293">
@@ -37031,7 +37031,7 @@
         <v>15.65</v>
       </c>
       <c r="C293" t="n">
-        <v>-8.376899999999999</v>
+        <v>-10.7211</v>
       </c>
     </row>
     <row r="294">
@@ -37042,7 +37042,7 @@
         <v>15.65</v>
       </c>
       <c r="C294" t="n">
-        <v>-1.3345</v>
+        <v>-6.0327</v>
       </c>
     </row>
     <row r="295">
@@ -37053,7 +37053,7 @@
         <v>15.65</v>
       </c>
       <c r="C295" t="n">
-        <v>7.2623</v>
+        <v>3.3637</v>
       </c>
     </row>
     <row r="296">
@@ -37064,7 +37064,7 @@
         <v>15.65</v>
       </c>
       <c r="C296" t="n">
-        <v>11.9409</v>
+        <v>11.1608</v>
       </c>
     </row>
     <row r="297">
@@ -37075,7 +37075,7 @@
         <v>15.65</v>
       </c>
       <c r="C297" t="n">
-        <v>13.6949</v>
+        <v>12.721</v>
       </c>
     </row>
     <row r="298">
@@ -37086,7 +37086,7 @@
         <v>15.65</v>
       </c>
       <c r="C298" t="n">
-        <v>14.7086</v>
+        <v>14.6687</v>
       </c>
     </row>
     <row r="299">
@@ -37097,7 +37097,7 @@
         <v>-15.65</v>
       </c>
       <c r="C299" t="n">
-        <v>11.5235</v>
+        <v>14.7485</v>
       </c>
     </row>
     <row r="300">
@@ -37108,7 +37108,7 @@
         <v>-15.65</v>
       </c>
       <c r="C300" t="n">
-        <v>2.5189</v>
+        <v>8.298400000000001</v>
       </c>
     </row>
     <row r="301">
@@ -37119,7 +37119,7 @@
         <v>-15.65</v>
       </c>
       <c r="C301" t="n">
-        <v>-6.9655</v>
+        <v>-3.2606</v>
       </c>
     </row>
     <row r="302">
@@ -37130,7 +37130,7 @@
         <v>-15.65</v>
       </c>
       <c r="C302" t="n">
-        <v>-11.6733</v>
+        <v>-10.6703</v>
       </c>
     </row>
     <row r="303">
@@ -37141,7 +37141,7 @@
         <v>-15.65</v>
       </c>
       <c r="C303" t="n">
-        <v>-13.6381</v>
+        <v>-12.6763</v>
       </c>
     </row>
     <row r="304">
@@ -37152,7 +37152,7 @@
         <v>-15.65</v>
       </c>
       <c r="C304" t="n">
-        <v>-15.3832</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="305">
@@ -37163,7 +37163,7 @@
         <v>-15.65</v>
       </c>
       <c r="C305" t="n">
-        <v>-15.9034</v>
+        <v>-16.1664</v>
       </c>
     </row>
     <row r="306">
@@ -37174,7 +37174,7 @@
         <v>-15.65</v>
       </c>
       <c r="C306" t="n">
-        <v>-15.6932</v>
+        <v>-15.6403</v>
       </c>
     </row>
     <row r="307">
@@ -37185,7 +37185,7 @@
         <v>-15.65</v>
       </c>
       <c r="C307" t="n">
-        <v>-15.2437</v>
+        <v>-15.7461</v>
       </c>
     </row>
     <row r="308">
@@ -37196,7 +37196,7 @@
         <v>15.65</v>
       </c>
       <c r="C308" t="n">
-        <v>-12.8587</v>
+        <v>-14.7413</v>
       </c>
     </row>
     <row r="309">
@@ -37207,7 +37207,7 @@
         <v>15.65</v>
       </c>
       <c r="C309" t="n">
-        <v>-5.8971</v>
+        <v>-10.9761</v>
       </c>
     </row>
     <row r="310">
@@ -37218,7 +37218,7 @@
         <v>15.65</v>
       </c>
       <c r="C310" t="n">
-        <v>4.0174</v>
+        <v>-0.8179999999999999</v>
       </c>
     </row>
     <row r="311">
@@ -37229,7 +37229,7 @@
         <v>15.65</v>
       </c>
       <c r="C311" t="n">
-        <v>10.7831</v>
+        <v>8.8528</v>
       </c>
     </row>
     <row r="312">
@@ -37240,7 +37240,7 @@
         <v>15.65</v>
       </c>
       <c r="C312" t="n">
-        <v>13.6627</v>
+        <v>12.7135</v>
       </c>
     </row>
     <row r="313">
@@ -37251,7 +37251,7 @@
         <v>15.65</v>
       </c>
       <c r="C313" t="n">
-        <v>14.3773</v>
+        <v>14.6118</v>
       </c>
     </row>
     <row r="314">
@@ -37262,7 +37262,7 @@
         <v>15.65</v>
       </c>
       <c r="C314" t="n">
-        <v>14.9139</v>
+        <v>14.1427</v>
       </c>
     </row>
     <row r="315">
@@ -37273,7 +37273,7 @@
         <v>-15.65</v>
       </c>
       <c r="C315" t="n">
-        <v>8.822900000000001</v>
+        <v>15.6851</v>
       </c>
     </row>
     <row r="316">
@@ -37284,7 +37284,7 @@
         <v>-15.65</v>
       </c>
       <c r="C316" t="n">
-        <v>-2.3727</v>
+        <v>1.9608</v>
       </c>
     </row>
     <row r="317">
@@ -37295,7 +37295,7 @@
         <v>-15.65</v>
       </c>
       <c r="C317" t="n">
-        <v>-9.1477</v>
+        <v>-6.7061</v>
       </c>
     </row>
     <row r="318">
@@ -37306,7 +37306,7 @@
         <v>15.65</v>
       </c>
       <c r="C318" t="n">
-        <v>-9.8247</v>
+        <v>-11.5893</v>
       </c>
     </row>
     <row r="319">
@@ -37317,7 +37317,7 @@
         <v>15.65</v>
       </c>
       <c r="C319" t="n">
-        <v>-3.36</v>
+        <v>-8.0601</v>
       </c>
     </row>
     <row r="320">
@@ -37328,7 +37328,7 @@
         <v>15.65</v>
       </c>
       <c r="C320" t="n">
-        <v>5.069</v>
+        <v>1.3402</v>
       </c>
     </row>
     <row r="321">
@@ -37339,7 +37339,7 @@
         <v>-15.65</v>
       </c>
       <c r="C321" t="n">
-        <v>5.4773</v>
+        <v>8.7979</v>
       </c>
     </row>
     <row r="322">
@@ -37350,7 +37350,7 @@
         <v>-15.65</v>
       </c>
       <c r="C322" t="n">
-        <v>-2.1477</v>
+        <v>2.1566</v>
       </c>
     </row>
     <row r="323">
@@ -37361,7 +37361,7 @@
         <v>-15.65</v>
       </c>
       <c r="C323" t="n">
-        <v>-8.920299999999999</v>
+        <v>-6.4521</v>
       </c>
     </row>
     <row r="324">
@@ -37372,7 +37372,7 @@
         <v>-15.65</v>
       </c>
       <c r="C324" t="n">
-        <v>-13.1058</v>
+        <v>-11.3885</v>
       </c>
     </row>
     <row r="325">
@@ -37383,7 +37383,7 @@
         <v>-15.65</v>
       </c>
       <c r="C325" t="n">
-        <v>-14.7468</v>
+        <v>-14.8232</v>
       </c>
     </row>
     <row r="326">
@@ -37394,7 +37394,7 @@
         <v>-15.65</v>
       </c>
       <c r="C326" t="n">
-        <v>-12.3319</v>
+        <v>-14.6703</v>
       </c>
     </row>
     <row r="327">
@@ -37405,7 +37405,7 @@
         <v>15.65</v>
       </c>
       <c r="C327" t="n">
-        <v>-4.3616</v>
+        <v>-9.993399999999999</v>
       </c>
     </row>
     <row r="328">
@@ -37416,7 +37416,7 @@
         <v>15.65</v>
       </c>
       <c r="C328" t="n">
-        <v>5.1865</v>
+        <v>1.2703</v>
       </c>
     </row>
     <row r="329">
@@ -37427,7 +37427,7 @@
         <v>15.65</v>
       </c>
       <c r="C329" t="n">
-        <v>7.505</v>
+        <v>9.1028</v>
       </c>
     </row>
     <row r="330">
@@ -37438,7 +37438,7 @@
         <v>-15.65</v>
       </c>
       <c r="C330" t="n">
-        <v>1.1143</v>
+        <v>5.9072</v>
       </c>
     </row>
     <row r="331">
@@ -37449,7 +37449,7 @@
         <v>-15.65</v>
       </c>
       <c r="C331" t="n">
-        <v>-7.0735</v>
+        <v>-3.6786</v>
       </c>
     </row>
     <row r="332">
@@ -37460,7 +37460,7 @@
         <v>-15.65</v>
       </c>
       <c r="C332" t="n">
-        <v>-8.292</v>
+        <v>-10.4683</v>
       </c>
     </row>
     <row r="333">
@@ -37471,7 +37471,7 @@
         <v>15.65</v>
       </c>
       <c r="C333" t="n">
-        <v>-1.8675</v>
+        <v>-6.1158</v>
       </c>
     </row>
     <row r="334">
@@ -37482,7 +37482,7 @@
         <v>15.65</v>
       </c>
       <c r="C334" t="n">
-        <v>6.0744</v>
+        <v>2.3808</v>
       </c>
     </row>
     <row r="335">
@@ -37493,7 +37493,7 @@
         <v>15.65</v>
       </c>
       <c r="C335" t="n">
-        <v>11.6828</v>
+        <v>9.7681</v>
       </c>
     </row>
     <row r="336">
@@ -37504,7 +37504,7 @@
         <v>15.65</v>
       </c>
       <c r="C336" t="n">
-        <v>14.1207</v>
+        <v>13.5976</v>
       </c>
     </row>
     <row r="337">
@@ -37515,7 +37515,7 @@
         <v>15.65</v>
       </c>
       <c r="C337" t="n">
-        <v>14.6677</v>
+        <v>14.6438</v>
       </c>
     </row>
     <row r="338">
@@ -37526,7 +37526,7 @@
         <v>15.65</v>
       </c>
       <c r="C338" t="n">
-        <v>15.9113</v>
+        <v>14.6915</v>
       </c>
     </row>
     <row r="339">
@@ -37537,7 +37537,7 @@
         <v>15.65</v>
       </c>
       <c r="C339" t="n">
-        <v>15.9048</v>
+        <v>17.1311</v>
       </c>
     </row>
     <row r="340">
@@ -37548,7 +37548,7 @@
         <v>15.65</v>
       </c>
       <c r="C340" t="n">
-        <v>15.1716</v>
+        <v>14.6784</v>
       </c>
     </row>
     <row r="341">
@@ -37559,7 +37559,7 @@
         <v>15.65</v>
       </c>
       <c r="C341" t="n">
-        <v>14.2495</v>
+        <v>15.6648</v>
       </c>
     </row>
     <row r="342">
@@ -37570,7 +37570,7 @@
         <v>-15.65</v>
       </c>
       <c r="C342" t="n">
-        <v>8.420500000000001</v>
+        <v>12.8342</v>
       </c>
     </row>
     <row r="343">
@@ -37581,7 +37581,7 @@
         <v>-15.65</v>
       </c>
       <c r="C343" t="n">
-        <v>-1.4314</v>
+        <v>4.0068</v>
       </c>
     </row>
     <row r="344">
@@ -37592,7 +37592,7 @@
         <v>-15.65</v>
       </c>
       <c r="C344" t="n">
-        <v>-7.8204</v>
+        <v>-6.8695</v>
       </c>
     </row>
     <row r="345">
@@ -37603,7 +37603,7 @@
         <v>15.65</v>
       </c>
       <c r="C345" t="n">
-        <v>-4.0917</v>
+        <v>-8.7714</v>
       </c>
     </row>
     <row r="346">
@@ -37614,7 +37614,7 @@
         <v>15.65</v>
       </c>
       <c r="C346" t="n">
-        <v>3.9954</v>
+        <v>0.588</v>
       </c>
     </row>
     <row r="347">
@@ -37625,7 +37625,7 @@
         <v>15.65</v>
       </c>
       <c r="C347" t="n">
-        <v>9.8729</v>
+        <v>7.4029</v>
       </c>
     </row>
     <row r="348">
@@ -37636,7 +37636,7 @@
         <v>15.65</v>
       </c>
       <c r="C348" t="n">
-        <v>13.6907</v>
+        <v>12.3429</v>
       </c>
     </row>
     <row r="349">
@@ -37647,7 +37647,7 @@
         <v>15.65</v>
       </c>
       <c r="C349" t="n">
-        <v>15.2916</v>
+        <v>15.0386</v>
       </c>
     </row>
     <row r="350">
@@ -37658,7 +37658,7 @@
         <v>15.65</v>
       </c>
       <c r="C350" t="n">
-        <v>15.1657</v>
+        <v>15.5446</v>
       </c>
     </row>
     <row r="351">
@@ -37669,7 +37669,7 @@
         <v>15.65</v>
       </c>
       <c r="C351" t="n">
-        <v>15.1708</v>
+        <v>14.7869</v>
       </c>
     </row>
     <row r="352">
@@ -37680,7 +37680,7 @@
         <v>15.65</v>
       </c>
       <c r="C352" t="n">
-        <v>15.8986</v>
+        <v>15.5547</v>
       </c>
     </row>
     <row r="353">
@@ -37691,7 +37691,7 @@
         <v>15.65</v>
       </c>
       <c r="C353" t="n">
-        <v>15.4743</v>
+        <v>16.2425</v>
       </c>
     </row>
     <row r="354">
@@ -37702,7 +37702,7 @@
         <v>-15.65</v>
       </c>
       <c r="C354" t="n">
-        <v>9.4735</v>
+        <v>14.706</v>
       </c>
     </row>
     <row r="355">
@@ -37713,7 +37713,7 @@
         <v>-15.65</v>
       </c>
       <c r="C355" t="n">
-        <v>-0.5735</v>
+        <v>4.2409</v>
       </c>
     </row>
     <row r="356">
@@ -37724,7 +37724,7 @@
         <v>-15.65</v>
       </c>
       <c r="C356" t="n">
-        <v>-7.8952</v>
+        <v>-5.388</v>
       </c>
     </row>
     <row r="357">
@@ -37735,7 +37735,7 @@
         <v>-15.65</v>
       </c>
       <c r="C357" t="n">
-        <v>-12.5996</v>
+        <v>-10.4024</v>
       </c>
     </row>
     <row r="358">
@@ -37746,7 +37746,7 @@
         <v>-15.65</v>
       </c>
       <c r="C358" t="n">
-        <v>-14.7763</v>
+        <v>-14.7967</v>
       </c>
     </row>
     <row r="359">
@@ -37757,7 +37757,7 @@
         <v>-15.65</v>
       </c>
       <c r="C359" t="n">
-        <v>-14.7176</v>
+        <v>-14.7558</v>
       </c>
     </row>
     <row r="360">
@@ -37768,7 +37768,7 @@
         <v>15.65</v>
       </c>
       <c r="C360" t="n">
-        <v>-11.4351</v>
+        <v>-14.6793</v>
       </c>
     </row>
     <row r="361">
@@ -37779,7 +37779,7 @@
         <v>15.65</v>
       </c>
       <c r="C361" t="n">
-        <v>-2.5911</v>
+        <v>-8.190799999999999</v>
       </c>
     </row>
     <row r="362">
@@ -37790,7 +37790,7 @@
         <v>15.65</v>
       </c>
       <c r="C362" t="n">
-        <v>7.0746</v>
+        <v>3.0086</v>
       </c>
     </row>
     <row r="363">
@@ -37801,7 +37801,7 @@
         <v>15.65</v>
       </c>
       <c r="C363" t="n">
-        <v>11.9162</v>
+        <v>11.1407</v>
       </c>
     </row>
     <row r="364">
@@ -37812,7 +37812,7 @@
         <v>15.65</v>
       </c>
       <c r="C364" t="n">
-        <v>13.6746</v>
+        <v>12.6918</v>
       </c>
     </row>
     <row r="365">
@@ -37823,7 +37823,7 @@
         <v>15.65</v>
       </c>
       <c r="C365" t="n">
-        <v>14.6695</v>
+        <v>14.6574</v>
       </c>
     </row>
     <row r="366">
@@ -37834,7 +37834,7 @@
         <v>15.65</v>
       </c>
       <c r="C366" t="n">
-        <v>12.0024</v>
+        <v>14.6816</v>
       </c>
     </row>
     <row r="367">
@@ -37845,7 +37845,7 @@
         <v>-15.65</v>
       </c>
       <c r="C367" t="n">
-        <v>3.6508</v>
+        <v>9.3232</v>
       </c>
     </row>
     <row r="368">
@@ -37856,7 +37856,7 @@
         <v>-15.65</v>
       </c>
       <c r="C368" t="n">
-        <v>-5.8489</v>
+        <v>-2.0217</v>
       </c>
     </row>
     <row r="369">
@@ -37867,7 +37867,7 @@
         <v>-15.65</v>
       </c>
       <c r="C369" t="n">
-        <v>-11.152</v>
+        <v>-9.6761</v>
       </c>
     </row>
     <row r="370">
@@ -37878,7 +37878,7 @@
         <v>-15.65</v>
       </c>
       <c r="C370" t="n">
-        <v>-13.6013</v>
+        <v>-12.6278</v>
       </c>
     </row>
     <row r="371">
@@ -37889,7 +37889,7 @@
         <v>-15.65</v>
       </c>
       <c r="C371" t="n">
-        <v>-14.6331</v>
+        <v>-14.5747</v>
       </c>
     </row>
     <row r="372">
@@ -37900,7 +37900,7 @@
         <v>-15.65</v>
       </c>
       <c r="C372" t="n">
-        <v>-13.446</v>
+        <v>-14.6915</v>
       </c>
     </row>
     <row r="373">
@@ -37911,7 +37911,7 @@
         <v>15.65</v>
       </c>
       <c r="C373" t="n">
-        <v>-6.2493</v>
+        <v>-12.2006</v>
       </c>
     </row>
     <row r="374">
@@ -37922,7 +37922,7 @@
         <v>15.65</v>
       </c>
       <c r="C374" t="n">
-        <v>4.0611</v>
+        <v>-0.2979</v>
       </c>
     </row>
     <row r="375">
@@ -37933,7 +37933,7 @@
         <v>15.65</v>
       </c>
       <c r="C375" t="n">
-        <v>9.078799999999999</v>
+        <v>8.420199999999999</v>
       </c>
     </row>
     <row r="376">
@@ -37944,7 +37944,7 @@
         <v>-15.65</v>
       </c>
       <c r="C376" t="n">
-        <v>5.7384</v>
+        <v>9.737500000000001</v>
       </c>
     </row>
     <row r="377">
@@ -37955,7 +37955,7 @@
         <v>-15.65</v>
       </c>
       <c r="C377" t="n">
-        <v>-2.5955</v>
+        <v>1.7393</v>
       </c>
     </row>
     <row r="378">
@@ -37966,7 +37966,7 @@
         <v>-15.65</v>
       </c>
       <c r="C378" t="n">
-        <v>-7.7698</v>
+        <v>-6.9304</v>
       </c>
     </row>
     <row r="379">
@@ -37977,7 +37977,7 @@
         <v>15.65</v>
       </c>
       <c r="C379" t="n">
-        <v>-4.0118</v>
+        <v>-8.609299999999999</v>
       </c>
     </row>
     <row r="380">
@@ -37988,7 +37988,7 @@
         <v>15.65</v>
       </c>
       <c r="C380" t="n">
-        <v>4.4489</v>
+        <v>0.5857</v>
       </c>
     </row>
     <row r="381">
@@ -37999,7 +37999,7 @@
         <v>15.65</v>
       </c>
       <c r="C381" t="n">
-        <v>8.537800000000001</v>
+        <v>8.312099999999999</v>
       </c>
     </row>
     <row r="382">
@@ -38010,7 +38010,7 @@
         <v>-15.65</v>
       </c>
       <c r="C382" t="n">
-        <v>2.8105</v>
+        <v>8.763400000000001</v>
       </c>
     </row>
     <row r="383">
@@ -38021,7 +38021,7 @@
         <v>-15.65</v>
       </c>
       <c r="C383" t="n">
-        <v>-3.8932</v>
+        <v>-3.1423</v>
       </c>
     </row>
     <row r="384">
@@ -38032,7 +38032,7 @@
         <v>-15.65</v>
       </c>
       <c r="C384" t="n">
-        <v>-7.5556</v>
+        <v>-4.644</v>
       </c>
     </row>
     <row r="385">
@@ -38043,7 +38043,7 @@
         <v>15.65</v>
       </c>
       <c r="C385" t="n">
-        <v>-6.5251</v>
+        <v>-10.4673</v>
       </c>
     </row>
     <row r="386">
@@ -38054,7 +38054,7 @@
         <v>15.65</v>
       </c>
       <c r="C386" t="n">
-        <v>1.7298</v>
+        <v>-2.5829</v>
       </c>
     </row>
     <row r="387">
@@ -38065,7 +38065,7 @@
         <v>15.65</v>
       </c>
       <c r="C387" t="n">
-        <v>8.587899999999999</v>
+        <v>6.0425</v>
       </c>
     </row>
     <row r="388">
@@ -38076,7 +38076,7 @@
         <v>-15.65</v>
       </c>
       <c r="C388" t="n">
-        <v>7.3067</v>
+        <v>11.1332</v>
       </c>
     </row>
     <row r="389">
@@ -38087,7 +38087,7 @@
         <v>-15.65</v>
       </c>
       <c r="C389" t="n">
-        <v>-1.4218</v>
+        <v>3.4801</v>
       </c>
     </row>
     <row r="390">

</xml_diff>